<commit_message>
fix(bar-checklists-en): ronda 1 de la revisión adversarial — 6 MAYOR + 16 menor aplicados
Sin 2-for-1 ni barra libre pública, Shelf life, tiras de sanitizante, nada de rellenar botellas de licor
(26 U.S.C. 5301(c)), ID 21+ y no servir a visiblemente ebrios en bartender y cocktail server, calendario US
corregido, party pump, aviso de alérgenos FDA 3-602.12(C). G1-G8 verdes, autotest 16/16; base idéntico.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/bar-checklist-templates/01-bar-opening-closing-checklists.xlsx
+++ b/astro-site/public/dl/bar-checklist-templates/01-bar-opening-closing-checklists.xlsx
@@ -1085,7 +1085,7 @@
       </c>
       <c r="B7" s="40" t="inlineStr">
         <is>
-          <t>No hand/arm jewelry except a plain band; nails short, clean, no polish or acrylics; no bare-hand contact with ice, citrus or garnish: use tongs, picks, a scoop or gloves</t>
+          <t>No hand/arm jewelry except a plain band; nails short, clean, no polish or acrylics; no bare-hand contact with ice, citrus or garnish (FDA Food Code 3-301.11): use tongs, picks, a scoop or gloves</t>
         </is>
       </c>
       <c r="C7" s="41" t="inlineStr">
@@ -2376,7 +2376,7 @@
       </c>
       <c r="B15" s="40" t="inlineStr">
         <is>
-          <t>Sanitize the bar top</t>
+          <t>Sanitize the bar top; test the sanitizer with strips (ppm on the label)</t>
         </is>
       </c>
       <c r="C15" s="41" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="B24" s="40" t="inlineStr">
         <is>
-          <t>Check that the day's cash count is closed and signed: it is not repeated here, it is done on "Cash Drawer Closing" in 09-cash-drawer-opening-closing.xlsx</t>
+          <t>Close out every open tab (no open checks before the Z report) and check that the day's cash count is closed and signed: it is not repeated here, it is done on "Cash Drawer Closing" in 09-cash-drawer-opening-closing.xlsx</t>
         </is>
       </c>
       <c r="C24" s="41" t="inlineStr">

</xml_diff>